<commit_message>
feat(users,interviews): colonnes d'import en français, contrainte manager RH, date/lieu entretien
- import_csv utilisateurs : en-têtes CSV en français (Prénom, Nom, Matricule,
  Email, Sexe, etc.), templates xlsx mis à jour en conséquence ; retire les
  colonnes Salaire brut mensuel et Tickets restaurant du template utilisateurs
- un utilisateur au rôle RH ne peut plus avoir de manager, et ne peut plus être
  désigné comme manager (N+1) d'un autre utilisateur ; masque le champ N+1
  dans le formulaire utilisateur quand le rôle est RH
- fix : User.__str__ plantait si email est vide (email désormais nullable)
- entretien : la date de réalisation (calendrier) est déplacée dans la carte
  "Informations générales" ; le champ Lieu affiche désormais le site du
  manager plutôt que celui du collaborateur
</commit_message>
<xml_diff>
--- a/doc/template_utilisateurs.xlsx
+++ b/doc/template_utilisateurs.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -425,116 +425,104 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>first_name</t>
+          <t>Prénom</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>last_name</t>
+          <t>Nom</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>matricule</t>
+          <t>Matricule</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>sexe</t>
+          <t>Sexe</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>date_naissance</t>
+          <t>Date de naissance</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>telephone</t>
+          <t>Téléphone</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>hire_date</t>
+          <t>Date d'embauche</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>date_sortie</t>
+          <t>Date de sortie</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>type_contrat</t>
+          <t>Type contrat</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>coefficient</t>
+          <t>Coefficient</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>salaire_brut</t>
+          <t>Rôle</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>service</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>Matricule N+1</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>manager_matricule</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>forfait_jour</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>tickets_restaurant</t>
+          <t>Forfait jour</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(doc): retire la colonne Forfait jour du template xlsx utilisateurs
</commit_message>
<xml_diff>
--- a/doc/template_utilisateurs.xlsx
+++ b/doc/template_utilisateurs.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -436,7 +436,6 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,11 +517,6 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Matricule N+1</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Forfait jour</t>
         </is>
       </c>
     </row>

</xml_diff>